<commit_message>
Wire results to Lookskart products and persist quiz/consultation leads.
Replace Live Love Locks cart links with Lookskart PDPs and packshots, export brand catalogs, and save quiz emails plus consultation requests locally with a booking confirmation modal.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/docs/lookskart-hair-brands.xlsx
+++ b/docs/lookskart-hair-brands.xlsx
@@ -3,7 +3,7 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
   <workbookPr codeName="ThisWorkbook"/>
   <sheets>
-    <sheet name="Hair Brands" sheetId="1" r:id="rId1"/>
+    <sheet name="Focus Brands" sheetId="1" r:id="rId1"/>
     <sheet name="Notes" sheetId="2" r:id="rId2"/>
   </sheets>
 </workbook>
@@ -398,15 +398,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:F18"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
-    <col min="2" max="2" width="30.83203125" customWidth="1"/>
-    <col min="3" max="3" width="30.83203125" customWidth="1"/>
-    <col min="4" max="4" width="34.83203125" customWidth="1"/>
-    <col min="5" max="5" width="22.83203125" customWidth="1"/>
-    <col min="6" max="6" width="72.83203125" customWidth="1"/>
-    <col min="7" max="7" width="58.83203125" customWidth="1"/>
+    <col min="2" max="2" width="24.83203125" customWidth="1"/>
+    <col min="3" max="3" width="20.83203125" customWidth="1"/>
+    <col min="4" max="4" width="16.83203125" customWidth="1"/>
+    <col min="5" max="5" width="78.83203125" customWidth="1"/>
+    <col min="6" max="6" width="34.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -417,18 +416,15 @@
         <v>Brand</v>
       </c>
       <c r="C1" t="str">
-        <v>Category</v>
+        <v>Products on Lookskart</v>
       </c>
       <c r="D1" t="str">
-        <v>Focus</v>
+        <v>Has products now</v>
       </c>
       <c r="E1" t="str">
-        <v>Has products now</v>
+        <v>Collection URL</v>
       </c>
       <c r="F1" t="str">
-        <v>Collection URL</v>
-      </c>
-      <c r="G1" t="str">
         <v>Source</v>
       </c>
     </row>
@@ -437,22 +433,19 @@
         <v>1</v>
       </c>
       <c r="B2" t="str">
-        <v>Balmain</v>
-      </c>
-      <c r="C2" t="str">
-        <v>Hair Care &amp; Finish</v>
+        <v>Biotop</v>
+      </c>
+      <c r="C2">
+        <v>15</v>
       </c>
       <c r="D2" t="str">
-        <v>Hair care &amp; styling</v>
+        <v>Yes</v>
       </c>
       <c r="E2" t="str">
-        <v>No (empty collection)</v>
+        <v>https://lookskart.com/collections/biotop</v>
       </c>
       <c r="F2" t="str">
-        <v>https://lookskart.com/collections/balmain</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Brand menu &gt; Hair Care &amp; Finish</v>
+        <v>Lookskart live catalog export</v>
       </c>
     </row>
     <row r="3">
@@ -460,22 +453,19 @@
         <v>2</v>
       </c>
       <c r="B3" t="str">
-        <v>Biotop</v>
-      </c>
-      <c r="C3" t="str">
-        <v>Hair Care &amp; Finish</v>
+        <v>Brasil Cacau</v>
+      </c>
+      <c r="C3">
+        <v>8</v>
       </c>
       <c r="D3" t="str">
-        <v>Hair care (shampoo / treatments)</v>
+        <v>Yes</v>
       </c>
       <c r="E3" t="str">
-        <v>Yes</v>
+        <v>https://lookskart.com/collections/brasil-cacau</v>
       </c>
       <c r="F3" t="str">
-        <v>https://lookskart.com/collections/biotop</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Brand menu &gt; Hair Care &amp; Finish; Shop by Brand; Brand filter</v>
+        <v>Lookskart live catalog export</v>
       </c>
     </row>
     <row r="4">
@@ -483,22 +473,19 @@
         <v>3</v>
       </c>
       <c r="B4" t="str">
-        <v>Brasil Cacau</v>
-      </c>
-      <c r="C4" t="str">
-        <v>Hair Care &amp; Finish</v>
+        <v>Kerastase</v>
+      </c>
+      <c r="C4">
+        <v>63</v>
       </c>
       <c r="D4" t="str">
-        <v>Hair care / keratin treatments</v>
+        <v>Yes</v>
       </c>
       <c r="E4" t="str">
-        <v>Yes</v>
+        <v>https://lookskart.com/collections/kerastase</v>
       </c>
       <c r="F4" t="str">
-        <v>https://lookskart.com/collections/brasil-cacau</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Brand menu &gt; Hair Care &amp; Finish; Shop by Brand</v>
+        <v>Lookskart live catalog export</v>
       </c>
     </row>
     <row r="5">
@@ -506,22 +493,19 @@
         <v>4</v>
       </c>
       <c r="B5" t="str">
-        <v>Global Keratin</v>
-      </c>
-      <c r="C5" t="str">
-        <v>Hair Care &amp; Finish</v>
+        <v>K18</v>
+      </c>
+      <c r="C5">
+        <v>2</v>
       </c>
       <c r="D5" t="str">
-        <v>Hair care / keratin</v>
+        <v>Yes</v>
       </c>
       <c r="E5" t="str">
-        <v>Yes</v>
+        <v>https://lookskart.com/collections/k18</v>
       </c>
       <c r="F5" t="str">
-        <v>https://lookskart.com/collections/global-keratin</v>
-      </c>
-      <c r="G5" t="str">
-        <v>Brand menu &gt; Hair Care &amp; Finish; Shop by Brand</v>
+        <v>Lookskart live catalog export</v>
       </c>
     </row>
     <row r="6">
@@ -529,22 +513,19 @@
         <v>5</v>
       </c>
       <c r="B6" t="str">
-        <v>Kerastase</v>
-      </c>
-      <c r="C6" t="str">
-        <v>Hair Care &amp; Finish</v>
+        <v>L'Oreal Professionnel</v>
+      </c>
+      <c r="C6">
+        <v>53</v>
       </c>
       <c r="D6" t="str">
-        <v>Professional luxury hair care</v>
+        <v>Yes</v>
       </c>
       <c r="E6" t="str">
-        <v>Yes</v>
+        <v>https://lookskart.com/collections/loreal-professional</v>
       </c>
       <c r="F6" t="str">
-        <v>https://lookskart.com/collections/kerastase</v>
-      </c>
-      <c r="G6" t="str">
-        <v>Shop by Brand; Brand filter; Hair Care bestsellers</v>
+        <v>Lookskart live catalog export</v>
       </c>
     </row>
     <row r="7">
@@ -552,22 +533,19 @@
         <v>6</v>
       </c>
       <c r="B7" t="str">
-        <v>Kevin Murphy</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Hair Care &amp; Finish</v>
+        <v>Lea Levett</v>
+      </c>
+      <c r="C7">
+        <v>6</v>
       </c>
       <c r="D7" t="str">
-        <v>Hair care &amp; styling</v>
+        <v>Yes</v>
       </c>
       <c r="E7" t="str">
-        <v>No (empty collection)</v>
+        <v>https://lookskart.com/collections/lea-levett</v>
       </c>
       <c r="F7" t="str">
-        <v>https://lookskart.com/collections/kevin-murphy</v>
-      </c>
-      <c r="G7" t="str">
-        <v>Brand menu &gt; Hair Care &amp; Finish; Shop by Brand</v>
+        <v>Lookskart live catalog export</v>
       </c>
     </row>
     <row r="8">
@@ -575,22 +553,19 @@
         <v>7</v>
       </c>
       <c r="B8" t="str">
-        <v>K18</v>
-      </c>
-      <c r="C8" t="str">
-        <v>Hair Care &amp; Finish</v>
+        <v>Moroccanoil</v>
+      </c>
+      <c r="C8">
+        <v>21</v>
       </c>
       <c r="D8" t="str">
-        <v>Hair repair / treatment</v>
+        <v>Yes</v>
       </c>
       <c r="E8" t="str">
-        <v>Yes</v>
+        <v>https://lookskart.com/collections/moroccan-oil-hair</v>
       </c>
       <c r="F8" t="str">
-        <v>https://lookskart.com/collections/k18</v>
-      </c>
-      <c r="G8" t="str">
-        <v>Brand menu &gt; Hair Care &amp; Finish; Shop by Brand</v>
+        <v>Lookskart live catalog export</v>
       </c>
     </row>
     <row r="9">
@@ -598,22 +573,19 @@
         <v>8</v>
       </c>
       <c r="B9" t="str">
-        <v>L'Oreal Professionnel</v>
-      </c>
-      <c r="C9" t="str">
-        <v>Hair Care &amp; Finish</v>
+        <v>Olaplex</v>
+      </c>
+      <c r="C9">
+        <v>0</v>
       </c>
       <c r="D9" t="str">
-        <v>Hair care &amp; styling</v>
+        <v>No</v>
       </c>
       <c r="E9" t="str">
-        <v>Yes</v>
+        <v>https://lookskart.com/collections/olaplex</v>
       </c>
       <c r="F9" t="str">
-        <v>https://lookskart.com/collections/loreal-professional</v>
-      </c>
-      <c r="G9" t="str">
-        <v>Brand menu &gt; Hair Care &amp; Finish; Shop by Brand; Brand filter</v>
+        <v>Lookskart live catalog export</v>
       </c>
     </row>
     <row r="10">
@@ -621,22 +593,19 @@
         <v>9</v>
       </c>
       <c r="B10" t="str">
-        <v>Lea Levett</v>
-      </c>
-      <c r="C10" t="str">
-        <v>Hair Care &amp; Finish</v>
+        <v>Root Deep</v>
+      </c>
+      <c r="C10">
+        <v>1</v>
       </c>
       <c r="D10" t="str">
-        <v>Hair care</v>
+        <v>Yes</v>
       </c>
       <c r="E10" t="str">
-        <v>Yes</v>
+        <v>https://lookskart.com/collections/root-deep</v>
       </c>
       <c r="F10" t="str">
-        <v>https://lookskart.com/collections/lea-levett</v>
-      </c>
-      <c r="G10" t="str">
-        <v>Brand menu &gt; Hair Care &amp; Finish; Shop by Brand; Brand filter</v>
+        <v>Lookskart live catalog export</v>
       </c>
     </row>
     <row r="11">
@@ -644,22 +613,19 @@
         <v>10</v>
       </c>
       <c r="B11" t="str">
-        <v>Moroccanoil (Moroccan Oil Hair)</v>
-      </c>
-      <c r="C11" t="str">
-        <v>Hair Care &amp; Finish</v>
+        <v>Schwarzkopf</v>
+      </c>
+      <c r="C11">
+        <v>14</v>
       </c>
       <c r="D11" t="str">
-        <v>Hair care &amp; oil</v>
+        <v>Yes</v>
       </c>
       <c r="E11" t="str">
-        <v>Yes</v>
+        <v>https://lookskart.com/collections/schwarzkopfprof-professional</v>
       </c>
       <c r="F11" t="str">
-        <v>https://lookskart.com/collections/moroccan-oil-hair</v>
-      </c>
-      <c r="G11" t="str">
-        <v>Brand menu &gt; Hair Care &amp; Finish; Brand filter (Moroccanoil)</v>
+        <v>Lookskart live catalog export</v>
       </c>
     </row>
     <row r="12">
@@ -667,22 +633,19 @@
         <v>11</v>
       </c>
       <c r="B12" t="str">
-        <v>Olaplex</v>
-      </c>
-      <c r="C12" t="str">
-        <v>Hair Care &amp; Finish</v>
+        <v>18.21 Man Made</v>
+      </c>
+      <c r="C12">
+        <v>9</v>
       </c>
       <c r="D12" t="str">
-        <v>Bond-building hair care</v>
+        <v>Yes</v>
       </c>
       <c r="E12" t="str">
-        <v>No (empty collection)</v>
+        <v>https://lookskart.com/collections/18-21-man</v>
       </c>
       <c r="F12" t="str">
-        <v>https://lookskart.com/collections/olaplex</v>
-      </c>
-      <c r="G12" t="str">
-        <v>Brand menu &gt; Hair Care &amp; Finish; Shop by Brand</v>
+        <v>Lookskart live catalog export</v>
       </c>
     </row>
     <row r="13">
@@ -690,22 +653,19 @@
         <v>12</v>
       </c>
       <c r="B13" t="str">
-        <v>Rene Furturer</v>
-      </c>
-      <c r="C13" t="str">
-        <v>Hair Care &amp; Finish</v>
+        <v>TAILOR'S</v>
+      </c>
+      <c r="C13">
+        <v>13</v>
       </c>
       <c r="D13" t="str">
-        <v>Hair care</v>
+        <v>Yes</v>
       </c>
       <c r="E13" t="str">
-        <v>No (empty collection)</v>
+        <v>https://lookskart.com/collections/tailors-product-collection-for-whatsapp-wati</v>
       </c>
       <c r="F13" t="str">
-        <v>https://lookskart.com/collections/rene-furturer</v>
-      </c>
-      <c r="G13" t="str">
-        <v>Brand menu &gt; Hair Care &amp; Finish; Shop by Brand</v>
+        <v>Lookskart live catalog export</v>
       </c>
     </row>
     <row r="14">
@@ -713,22 +673,19 @@
         <v>13</v>
       </c>
       <c r="B14" t="str">
-        <v>Root Deep</v>
-      </c>
-      <c r="C14" t="str">
-        <v>Hair Care &amp; Finish</v>
+        <v>Wet Brush</v>
+      </c>
+      <c r="C14">
+        <v>0</v>
       </c>
       <c r="D14" t="str">
-        <v>Hair care</v>
+        <v>No</v>
       </c>
       <c r="E14" t="str">
-        <v>Yes</v>
+        <v>https://lookskart.com/collections/wet-brush</v>
       </c>
       <c r="F14" t="str">
-        <v>https://lookskart.com/collections/root-deep</v>
-      </c>
-      <c r="G14" t="str">
-        <v>Brand menu &gt; Hair Care &amp; Finish; Shop by Brand; Brand filter</v>
+        <v>Lookskart live catalog export</v>
       </c>
     </row>
     <row r="15">
@@ -736,22 +693,19 @@
         <v>14</v>
       </c>
       <c r="B15" t="str">
-        <v>Schwarzkopf Professional</v>
-      </c>
-      <c r="C15" t="str">
-        <v>Hair Care &amp; Finish</v>
+        <v>Let's Shave</v>
+      </c>
+      <c r="C15">
+        <v>8</v>
       </c>
       <c r="D15" t="str">
-        <v>Hair care &amp; styling</v>
+        <v>Yes</v>
       </c>
       <c r="E15" t="str">
-        <v>Yes</v>
+        <v>https://lookskart.com/collections/lets-shave</v>
       </c>
       <c r="F15" t="str">
-        <v>https://lookskart.com/collections/schwarzkopfprof-professional</v>
-      </c>
-      <c r="G15" t="str">
-        <v>Brand menu &gt; Hair Care &amp; Finish; Shop by Brand; Brand filter</v>
+        <v>Lookskart live catalog export</v>
       </c>
     </row>
     <row r="16">
@@ -759,22 +713,19 @@
         <v>15</v>
       </c>
       <c r="B16" t="str">
-        <v>American Crew</v>
-      </c>
-      <c r="C16" t="str">
-        <v>Mens / Tools &amp; Accessories</v>
+        <v>Redken</v>
+      </c>
+      <c r="C16">
+        <v>0</v>
       </c>
       <c r="D16" t="str">
-        <v>Mens hair styling &amp; care</v>
+        <v>No</v>
       </c>
       <c r="E16" t="str">
-        <v>No (empty collection)</v>
+        <v>https://lookskart.com/search?q=redken&amp;type=product</v>
       </c>
       <c r="F16" t="str">
-        <v>https://lookskart.com/collections/american-crew</v>
-      </c>
-      <c r="G16" t="str">
-        <v>Brand menu &gt; Mens, Tools &amp; Accessories; Shop by Brand</v>
+        <v>Lookskart live catalog export</v>
       </c>
     </row>
     <row r="17">
@@ -782,22 +733,19 @@
         <v>16</v>
       </c>
       <c r="B17" t="str">
-        <v>18.21 Man Made</v>
-      </c>
-      <c r="C17" t="str">
-        <v>Mens / Tools &amp; Accessories</v>
+        <v>Agnaya</v>
+      </c>
+      <c r="C17">
+        <v>0</v>
       </c>
       <c r="D17" t="str">
-        <v>Mens hair styling &amp; grooming</v>
+        <v>No</v>
       </c>
       <c r="E17" t="str">
-        <v>Yes</v>
+        <v>https://lookskart.com/search?q=agnaya&amp;type=product</v>
       </c>
       <c r="F17" t="str">
-        <v>https://lookskart.com/collections/18-21-man</v>
-      </c>
-      <c r="G17" t="str">
-        <v>Brand menu &gt; Mens, Tools &amp; Accessories</v>
+        <v>Lookskart live catalog export</v>
       </c>
     </row>
     <row r="18">
@@ -805,128 +753,33 @@
         <v>17</v>
       </c>
       <c r="B18" t="str">
-        <v>TAILOR'S</v>
-      </c>
-      <c r="C18" t="str">
-        <v>Mens Hair / Beard (featured)</v>
+        <v>pH Plex (Phplex)</v>
+      </c>
+      <c r="C18">
+        <v>3</v>
       </c>
       <c r="D18" t="str">
-        <v>Mens hair, beard &amp; styling</v>
+        <v>Yes</v>
       </c>
       <c r="E18" t="str">
-        <v>Yes</v>
+        <v>https://lookskart.com/search?q=ph+plex&amp;type=product</v>
       </c>
       <c r="F18" t="str">
-        <v>https://lookskart.com/collections/tailors-product-collection-for-whatsapp-wati</v>
-      </c>
-      <c r="G18" t="str">
-        <v>Featured banners / Curated for Men</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="B19" t="str">
-        <v>Dyson</v>
-      </c>
-      <c r="C19" t="str">
-        <v>Mens / Tools &amp; Accessories</v>
-      </c>
-      <c r="D19" t="str">
-        <v>Hair tools (dryers / stylers)</v>
-      </c>
-      <c r="E19" t="str">
-        <v>No (empty collection)</v>
-      </c>
-      <c r="F19" t="str">
-        <v>https://lookskart.com/collections/dyson</v>
-      </c>
-      <c r="G19" t="str">
-        <v>Brand menu &gt; Mens, Tools &amp; Accessories; Shop by Brand</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20" t="str">
-        <v>Wahl</v>
-      </c>
-      <c r="C20" t="str">
-        <v>Mens / Tools &amp; Accessories</v>
-      </c>
-      <c r="D20" t="str">
-        <v>Hair clippers / trimmers</v>
-      </c>
-      <c r="E20" t="str">
-        <v>No (empty collection)</v>
-      </c>
-      <c r="F20" t="str">
-        <v>https://lookskart.com/collections/wahl</v>
-      </c>
-      <c r="G20" t="str">
-        <v>Brand menu &gt; Mens, Tools &amp; Accessories; Shop by Brand</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21" t="str">
-        <v>Wet Brush</v>
-      </c>
-      <c r="C21" t="str">
-        <v>Mens / Tools &amp; Accessories</v>
-      </c>
-      <c r="D21" t="str">
-        <v>Hair brushes</v>
-      </c>
-      <c r="E21" t="str">
-        <v>No (empty collection)</v>
-      </c>
-      <c r="F21" t="str">
-        <v>https://lookskart.com/collections/wet-brush</v>
-      </c>
-      <c r="G21" t="str">
-        <v>Brand menu &gt; Mens, Tools &amp; Accessories; Shop by Brand</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22" t="str">
-        <v>Lets Shave</v>
-      </c>
-      <c r="C22" t="str">
-        <v>Mens / Tools &amp; Accessories</v>
-      </c>
-      <c r="D22" t="str">
-        <v>Shaving / grooming (beard &amp; body)</v>
-      </c>
-      <c r="E22" t="str">
-        <v>Yes</v>
-      </c>
-      <c r="F22" t="str">
-        <v>https://lookskart.com/collections/lets-shave</v>
-      </c>
-      <c r="G22" t="str">
-        <v>Brand menu &gt; Mens, Tools &amp; Accessories; Brand filter</v>
+        <v>Lookskart live catalog export</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:G22"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:F18"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B9"/>
   <cols>
-    <col min="1" max="1" width="28.83203125" customWidth="1"/>
+    <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="110.83203125" customWidth="1"/>
   </cols>
   <sheetData>
@@ -943,44 +796,68 @@
         <v>Source site</v>
       </c>
       <c r="B2" t="str">
-        <v>https://lookskart.com/</v>
+        <v>https://lookskart.com</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
-        <v>Scraped on</v>
+        <v>Catalog dump</v>
       </c>
       <c r="B3" t="str">
-        <v>2026-08-08</v>
+        <v>docs/data/lookskart-products-page1.json</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
-        <v>Hair Care &amp; Finish brands</v>
+        <v>Scraped on</v>
       </c>
       <c r="B4" t="str">
-        <v>Core list from Brand &gt; Hair Care &amp; Finish, plus Kerastase from Shop by Brand / products</v>
+        <v>2026-08-10</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
-        <v>Excluded (skincare-only)</v>
+        <v>Catalog size</v>
       </c>
       <c r="B5" t="str">
-        <v>Dermalogica; L'aamis Organic; Moroccan Oil Skin; Pedilabs Alchemy Cure Cream</v>
+        <v>241 live products returned by Shopify products.json (page 1; page 2 empty)</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Empty collections</v>
+        <v>Added brands</v>
       </c>
       <c r="B6" t="str">
-        <v>Brand pages exist in nav/Shop by Brand but currently show no products: Balmain, Kevin Murphy, Olaplex, Rene Furturer, American Crew, Dyson, Wahl, Wet Brush</v>
+        <v>Redken, Agnaya, pH Plex (Phplex) — requested additions beyond the original focus list</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="str">
+        <v>Redken / Agnaya</v>
+      </c>
+      <c r="B7" t="str">
+        <v>No products or collections found in the live Lookskart catalog as of scrape date</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="str">
+        <v>Olaplex / Wet Brush</v>
+      </c>
+      <c r="B8" t="str">
+        <v>Brand collection pages exist but currently show no products; older Olaplex PDP URLs indexed by search return 404</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="str">
+        <v>pH Plex</v>
+      </c>
+      <c r="B9" t="str">
+        <v>Sold on Lookskart under Looks Kart vendor (search “pH Plex”); 3 products in catalog</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:B6"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:B9"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>